<commit_message>
- correct terminology for subregions; - activate timeseries usage; - correct rest sector consideration; - upper boundary in set&control
</commit_message>
<xml_diff>
--- a/input/Set_and_Control_Parameters.xlsx
+++ b/input/Set_and_Control_Parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Projekte\endemo_Projects\endemo-ENS\endemo_IND_world_branch\endemo\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58D5FFDC-7AD7-4001-B453-C55B6F0DFA0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EB2B050-531E-41AB-881C-47446772453C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1710" yWindow="1020" windowWidth="20175" windowHeight="13230" tabRatio="730" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="33600" yWindow="1440" windowWidth="20175" windowHeight="13230" tabRatio="730" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GeneralSettings" sheetId="1" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="133">
   <si>
     <t>Country</t>
   </si>
@@ -455,6 +455,9 @@
   </si>
   <si>
     <t>Last considered year</t>
+  </si>
+  <si>
+    <t>Production quantity upper limit (unit description)</t>
   </si>
 </sst>
 </file>
@@ -569,7 +572,7 @@
       <alignment horizontal="right"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -595,6 +598,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -764,11 +770,11 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp6.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" fmlaLink="$C$8" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" fmlaLink="$C$8" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp7.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" fmlaLink="$C$9" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" fmlaLink="$C$9" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp8.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1919,15 +1925,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>19050</xdr:colOff>
+          <xdr:colOff>9525</xdr:colOff>
           <xdr:row>0</xdr:row>
-          <xdr:rowOff>352425</xdr:rowOff>
+          <xdr:rowOff>561975</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>742950</xdr:colOff>
+          <xdr:colOff>733425</xdr:colOff>
           <xdr:row>2</xdr:row>
-          <xdr:rowOff>19050</xdr:rowOff>
+          <xdr:rowOff>38100</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -4735,7 +4741,7 @@
         <v>13</v>
       </c>
       <c r="C8" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D8" t="s">
         <v>25</v>
@@ -4749,7 +4755,7 @@
         <v>14</v>
       </c>
       <c r="C9" s="5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D9" t="s">
         <v>26</v>
@@ -5451,7 +5457,7 @@
     <col min="2" max="2" width="18.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="25.7109375" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.7109375" customWidth="1"/>
     <col min="6" max="6" width="22.28515625" customWidth="1"/>
     <col min="7" max="7" width="56.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.85546875" bestFit="1" customWidth="1"/>
@@ -5459,7 +5465,7 @@
     <col min="10" max="10" width="12.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="1" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>74</v>
       </c>
@@ -5472,8 +5478,8 @@
       <c r="D1" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>49</v>
+      <c r="E1" s="16" t="s">
+        <v>132</v>
       </c>
       <c r="F1" s="7" t="s">
         <v>77</v>
@@ -5502,9 +5508,7 @@
       <c r="D2">
         <v>0</v>
       </c>
-      <c r="E2" s="4">
-        <v>0</v>
-      </c>
+      <c r="E2" s="4"/>
       <c r="F2" s="9" t="s">
         <v>7</v>
       </c>
@@ -5532,9 +5536,7 @@
       <c r="D3">
         <v>0</v>
       </c>
-      <c r="E3" s="4">
-        <v>0</v>
-      </c>
+      <c r="E3" s="4"/>
       <c r="F3" s="9">
         <f>100-F5</f>
         <v>0</v>
@@ -5562,9 +5564,7 @@
       <c r="D4">
         <v>0</v>
       </c>
-      <c r="E4" s="4">
-        <v>0</v>
-      </c>
+      <c r="E4" s="4"/>
       <c r="F4" s="9" t="s">
         <v>7</v>
       </c>
@@ -5591,9 +5591,7 @@
       <c r="D5">
         <v>0</v>
       </c>
-      <c r="E5" s="4">
-        <v>0</v>
-      </c>
+      <c r="E5" s="4"/>
       <c r="F5">
         <v>100</v>
       </c>
@@ -5620,9 +5618,7 @@
       <c r="D6">
         <v>0</v>
       </c>
-      <c r="E6" s="4">
-        <v>0</v>
-      </c>
+      <c r="E6" s="4"/>
       <c r="F6" s="9" t="s">
         <v>7</v>
       </c>
@@ -5649,9 +5645,7 @@
       <c r="D7">
         <v>0</v>
       </c>
-      <c r="E7" s="4">
-        <v>0</v>
-      </c>
+      <c r="E7" s="4"/>
       <c r="F7" s="9" t="s">
         <v>7</v>
       </c>
@@ -5678,9 +5672,7 @@
       <c r="D8">
         <v>0</v>
       </c>
-      <c r="E8" s="4">
-        <v>0</v>
-      </c>
+      <c r="E8" s="4"/>
       <c r="F8" s="9">
         <v>70</v>
       </c>
@@ -5704,9 +5696,7 @@
       <c r="D9">
         <v>0</v>
       </c>
-      <c r="E9" s="4">
-        <v>0</v>
-      </c>
+      <c r="E9" s="4"/>
       <c r="F9" s="9">
         <f>100-F8</f>
         <v>30</v>
@@ -5731,9 +5721,7 @@
       <c r="D10">
         <v>0</v>
       </c>
-      <c r="E10" s="4">
-        <v>0</v>
-      </c>
+      <c r="E10" s="4"/>
       <c r="F10" s="9" t="s">
         <v>7</v>
       </c>
@@ -5760,9 +5748,7 @@
       <c r="D11">
         <v>0</v>
       </c>
-      <c r="E11" s="4">
-        <v>0</v>
-      </c>
+      <c r="E11" s="4"/>
       <c r="F11">
         <v>100</v>
       </c>
@@ -5789,9 +5775,7 @@
       <c r="D12">
         <v>0</v>
       </c>
-      <c r="E12" s="4">
-        <v>0</v>
-      </c>
+      <c r="E12" s="4"/>
       <c r="F12">
         <v>100</v>
       </c>
@@ -5818,9 +5802,7 @@
       <c r="D13">
         <v>0</v>
       </c>
-      <c r="E13" s="4">
-        <v>0</v>
-      </c>
+      <c r="E13" s="4"/>
       <c r="F13">
         <v>100</v>
       </c>
@@ -5847,9 +5829,7 @@
       <c r="D14">
         <v>0</v>
       </c>
-      <c r="E14" s="4">
-        <v>0</v>
-      </c>
+      <c r="E14" s="4"/>
       <c r="F14">
         <v>100</v>
       </c>
@@ -5877,7 +5857,7 @@
         <v>0</v>
       </c>
       <c r="E15" s="4">
-        <v>0</v>
+        <v>6.4399999999999999E-2</v>
       </c>
       <c r="F15">
         <v>100</v>
@@ -5906,7 +5886,7 @@
         <v>0</v>
       </c>
       <c r="E16" s="4">
-        <v>0</v>
+        <v>2.9000000000000001E-2</v>
       </c>
       <c r="F16">
         <v>100</v>
@@ -5934,9 +5914,7 @@
       <c r="D17">
         <v>0</v>
       </c>
-      <c r="E17" s="4">
-        <v>0</v>
-      </c>
+      <c r="E17" s="4"/>
       <c r="F17" s="9">
         <f>100-F11</f>
         <v>0</v>
@@ -5964,9 +5942,7 @@
       <c r="D18">
         <v>0</v>
       </c>
-      <c r="E18" s="4">
-        <v>0</v>
-      </c>
+      <c r="E18" s="4"/>
       <c r="F18" s="9">
         <f>100-F12</f>
         <v>0</v>
@@ -5994,9 +5970,7 @@
       <c r="D19">
         <v>0</v>
       </c>
-      <c r="E19" s="4">
-        <v>0</v>
-      </c>
+      <c r="E19" s="4"/>
       <c r="F19" s="9">
         <f>100-F13</f>
         <v>0</v>
@@ -6024,9 +5998,7 @@
       <c r="D20">
         <v>0</v>
       </c>
-      <c r="E20" s="4">
-        <v>0</v>
-      </c>
+      <c r="E20" s="4"/>
       <c r="F20" s="9">
         <f>100-F14</f>
         <v>0</v>
@@ -6055,7 +6027,8 @@
         <v>0</v>
       </c>
       <c r="E21" s="4">
-        <v>0</v>
+        <f>E15</f>
+        <v>6.4399999999999999E-2</v>
       </c>
       <c r="F21" s="9">
         <f>100-F15</f>
@@ -6086,7 +6059,8 @@
         <v>0</v>
       </c>
       <c r="E22" s="4">
-        <v>0</v>
+        <f>E16</f>
+        <v>2.9000000000000001E-2</v>
       </c>
       <c r="F22" s="9">
         <f t="shared" ref="F22" si="1">100-F16</f>
@@ -6115,9 +6089,7 @@
       <c r="D23">
         <v>0</v>
       </c>
-      <c r="E23" s="4">
-        <v>0</v>
-      </c>
+      <c r="E23" s="4"/>
       <c r="F23" s="9" t="s">
         <v>7</v>
       </c>
@@ -6144,9 +6116,7 @@
       <c r="D24">
         <v>0</v>
       </c>
-      <c r="E24" s="4">
-        <v>0</v>
-      </c>
+      <c r="E24" s="4"/>
       <c r="F24" s="9" t="s">
         <v>7</v>
       </c>
@@ -6173,9 +6143,7 @@
       <c r="D25">
         <v>0</v>
       </c>
-      <c r="E25" s="4">
-        <v>0.33</v>
-      </c>
+      <c r="E25" s="4"/>
       <c r="F25" s="9" t="s">
         <v>7</v>
       </c>
@@ -6203,9 +6171,7 @@
       <c r="D26" s="6">
         <v>0.7</v>
       </c>
-      <c r="E26" s="8">
-        <v>0.7</v>
-      </c>
+      <c r="E26" s="8"/>
       <c r="F26" s="10" t="s">
         <v>7</v>
       </c>
@@ -6226,12 +6192,13 @@
   <protectedRanges>
     <protectedRange sqref="F17:F22" name="Linked values"/>
   </protectedRanges>
-  <dataValidations count="5">
+  <dataValidations count="6">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Activate subsectors" prompt="Activate calculation and forecast of industrial subsectors._x000a_Unspecified subsector is automaticaly activated." sqref="B1" xr:uid="{949AC99B-8518-4C69-BDE9-CBF83CDC4BE9}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Show status" prompt="Shows status of industrial subsector activation" sqref="C1" xr:uid="{D39270FC-1E17-4BF1-A784-B322B986174F}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Production quantity development" prompt="User defined expectation for the yearly development from last available historical year or pregiven value till the forecasted year._x000a_To be applied with exponential function of production quantity extrapolation or if not enough data are available." sqref="D1" xr:uid="{B759DEDC-FFC7-4AED-960F-A7EC37EB9FCC}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Technology substitution" prompt="User defined expectation for the forecasted year" sqref="F1" xr:uid="{5BCC82F2-3048-4B59-9F52-5232CB2E59D7}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Prod. efficiency development" prompt="User defined expectation for the yearly change of the efficiency (applied on the pregiven value)_x000a_Applies only if the Trend calculation for specific energy requirements is disactivated." sqref="I1" xr:uid="{EA236F94-8106-431A-8B80-F2F9E2C16CB9}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Unit:" prompt="If calculation of the production quantity per capita is selected (see IND_general), then the unit is ton per capita._x000a_Otherwise, the unit is ton." sqref="E1" xr:uid="{C2BCDC4E-2C12-4FC3-BF03-7951C5B34506}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -6247,15 +6214,15 @@
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>1</xdr:col>
-                    <xdr:colOff>19050</xdr:colOff>
+                    <xdr:colOff>9525</xdr:colOff>
                     <xdr:row>0</xdr:row>
-                    <xdr:rowOff>352425</xdr:rowOff>
+                    <xdr:rowOff>561975</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>1</xdr:col>
-                    <xdr:colOff>742950</xdr:colOff>
+                    <xdr:colOff>733425</xdr:colOff>
                     <xdr:row>2</xdr:row>
-                    <xdr:rowOff>19050</xdr:rowOff>
+                    <xdr:rowOff>38100</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>

</xml_diff>